<commit_message>
Ignore generated datasets and add latest procurement records
</commit_message>
<xml_diff>
--- a/dados/enviadas/Editais.xlsx
+++ b/dados/enviadas/Editais.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="[$R$-416] #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="[$R$-416] #,##0.00"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -69,21 +70,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -451,375 +453,167 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="59" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>ITEM</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>MODALIDADE</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>VALOR_ESTIMADO</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>ORGAO</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>DATA_DISPUTA</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>PORTAL</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>LINK_PORTAL</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>LINK_PNCP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Editais</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>27/2026</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Serviços elétricos</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>97/2026-PE.70/2026/2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Kit lanches</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>198255.59</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>SERVICO SOCIAL DO COMERCIO - ADMINISTRACAO REGIONAL NO ESTADO DE MINAS GERAIS</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>13/10/2026</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>ComprasGov</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=92648305000272026</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/03643856000173/2026/64</t>
+      <c r="E2" s="5" t="n">
+        <v>702630.29</v>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE ITATIBA</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>46318.36805555555</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/50122571000177/2026/324</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Editais</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>113/2026</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Locação de beliches</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Dispensa</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>18793.13</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE SANTANA DE PARNAIBA</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Portal de Compras Públicas</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.portaldecompraspublicas.com.br/processos/SP/Prefeitura-Municipal-de-Santana-de-Parnaiba-1139/DE-113-2026-2026-514525</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/46522983000127/2026/356</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Editais</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>022/2026</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Geradores</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>21/2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Instalação de geradores</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>191314.5</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>CISALP-CONSORCIO PUBLICO INTERMUNICIPAL DE SAUDE A MICRO-REGIAO DO ALTO PARANAIBA</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Licitanet</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>https://licitanet.com.br/sessao/202583</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/02319394000170/2026/78</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Editais</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>16/2026</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Geradores</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Pregão - Eletrônico</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>71000</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE GOIANA</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>AMM Licita</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>https://app2.ammlicita.org.br/pesquisa/114808</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/01611137000145/2026/25</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Editais</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>132/2026</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Grupo gerador</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Pregão - Eletrônico</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>1269975.5</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>TRIBUNAL SUPERIOR ELEITORAL</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="E3" s="5" t="n">
+        <v>401043.77</v>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>SERVICO SOCIAL DO COMERCIO - ADMINISTRACAO REGIONAL NO ESTADO DE MINAS GERAIS</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>46310.375</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>ComprasGov</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=07001305001322026</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/00509018000113/2026/2151</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Editais</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>90/2026</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Geradores</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Pregão - Eletrônico</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>3821900.51</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>COMANDO DO EXERCITO</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>13/10/2026</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>ComprasGov</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=16036705000902026</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/00394452000103/2026/18565</t>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=92648305000212026</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/03643856000173/2026/61</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>